<commit_message>
Build Python data processing pipeline
</commit_message>
<xml_diff>
--- a/data/raw/zalando_raw_data.xlsx
+++ b/data/raw/zalando_raw_data.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nishtha/Desktop/projects/zalando-performance-intelligence/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71EEC764-BCD8-7A41-8348-E7D53542D44C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DE56F2A-4872-F649-A014-C25EA5095D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14260" yWindow="500" windowWidth="14160" windowHeight="15920" activeTab="2" xr2:uid="{A0F484E8-04F7-6E4B-B80A-EC377135022B}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="3" xr2:uid="{A0F484E8-04F7-6E4B-B80A-EC377135022B}"/>
   </bookViews>
   <sheets>
     <sheet name="financial_kpis" sheetId="1" r:id="rId1"/>
     <sheet name="operating_kpis" sheetId="2" r:id="rId2"/>
     <sheet name="sources" sheetId="3" r:id="rId3"/>
+    <sheet name="interim_kpis" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="109">
   <si>
     <t>period</t>
   </si>
@@ -69,6 +70,9 @@
     <t>free_cash_flow_eur_m</t>
   </si>
   <si>
+    <t>employees</t>
+  </si>
+  <si>
     <t>source_document</t>
   </si>
   <si>
@@ -99,12 +103,6 @@
     <t>document_type</t>
   </si>
   <si>
-    <t>publication_date</t>
-  </si>
-  <si>
-    <t>url</t>
-  </si>
-  <si>
     <t>local_filename</t>
   </si>
   <si>
@@ -138,18 +136,12 @@
     <t>orders_per_active_customer</t>
   </si>
   <si>
-    <t>average_employees</t>
-  </si>
-  <si>
     <t>segment</t>
   </si>
   <si>
     <t>Group</t>
   </si>
   <si>
-    <t>Includes ABOUT YOU following consolidation from 11 Jul 2025</t>
-  </si>
-  <si>
     <t>B2C</t>
   </si>
   <si>
@@ -168,9 +160,6 @@
     <t>Comparative segment figures as presented in Annual Report 2025</t>
   </si>
   <si>
-    <t>Customer metrics marked LTM where applicable; includes ABOUT YOU following consolidation from 11 Jul 2025</t>
-  </si>
-  <si>
     <t>primary_use</t>
   </si>
   <si>
@@ -183,13 +172,199 @@
     <t>zalando_annual_report_2025.pdf</t>
   </si>
   <si>
-    <t>PASTE_OFFICIAL_URL_HERE</t>
-  </si>
-  <si>
-    <t>Financial KPIs; operating KPIs; segment performance; KPI definitions; financial statements</t>
-  </si>
-  <si>
-    <t>Primary FY2025 source; contains FY2024 comparative figures</t>
+    <t>Includes ABOUT YOU following consolidation in 2025</t>
+  </si>
+  <si>
+    <t>FY2023</t>
+  </si>
+  <si>
+    <t>Zalando Annual Report 2024</t>
+  </si>
+  <si>
+    <t>Comparative figures as presented in Annual Report 2024</t>
+  </si>
+  <si>
+    <t>FY2022</t>
+  </si>
+  <si>
+    <t>Zalando Annual Report 2023</t>
+  </si>
+  <si>
+    <t>Comparative figures as presented in Annual Report 2023</t>
+  </si>
+  <si>
+    <t>FY2021</t>
+  </si>
+  <si>
+    <t>Zalando Annual Report 2022</t>
+  </si>
+  <si>
+    <t>Comparative figures as presented in Annual Report 2022</t>
+  </si>
+  <si>
+    <t>FY2020</t>
+  </si>
+  <si>
+    <t>Zalando Annual Report 2021</t>
+  </si>
+  <si>
+    <t>Comparative figures as presented in Annual Report 2021</t>
+  </si>
+  <si>
+    <t>FY2019</t>
+  </si>
+  <si>
+    <t>Zalando Annual Report 2020</t>
+  </si>
+  <si>
+    <t>Comparative figures as presented in Annual Report 2020</t>
+  </si>
+  <si>
+    <t>Customer metrics marked LTM where applicable; includes ABOUT YOU following consolidation</t>
+  </si>
+  <si>
+    <t>Comparative figures as presented in Annual Report 2020; GMV per active customer not shown in this key-figures table</t>
+  </si>
+  <si>
+    <t>FY2025 data; FY2024 comparatives; B2C/B2B segment reporting; definitions</t>
+  </si>
+  <si>
+    <t>Primary FY2025 source</t>
+  </si>
+  <si>
+    <t>SRC002</t>
+  </si>
+  <si>
+    <t>zalando_annual_report_2024.pdf</t>
+  </si>
+  <si>
+    <t>FY2024 reporting; FY2023 comparatives; strategy and segment reporting</t>
+  </si>
+  <si>
+    <t>Preferred source for FY2023 historical observations</t>
+  </si>
+  <si>
+    <t>SRC003</t>
+  </si>
+  <si>
+    <t>zalando_annual_report_2023.pdf</t>
+  </si>
+  <si>
+    <t>FY2023 reporting; FY2022 comparatives</t>
+  </si>
+  <si>
+    <t>Preferred source for FY2022 historical observations</t>
+  </si>
+  <si>
+    <t>SRC004</t>
+  </si>
+  <si>
+    <t>zalando_annual_report_2022.pdf</t>
+  </si>
+  <si>
+    <t>FY2022 reporting; FY2021 comparatives</t>
+  </si>
+  <si>
+    <t>Preferred source for FY2021 historical observations</t>
+  </si>
+  <si>
+    <t>SRC005</t>
+  </si>
+  <si>
+    <t>zalando_annual_report_2021.pdf</t>
+  </si>
+  <si>
+    <t>FY2021 reporting; FY2020 comparatives</t>
+  </si>
+  <si>
+    <t>Preferred source for FY2020 historical observations</t>
+  </si>
+  <si>
+    <t>SRC006</t>
+  </si>
+  <si>
+    <t>zalando_annual_report_2020.pdf</t>
+  </si>
+  <si>
+    <t>FY2020 reporting; FY2019 comparatives</t>
+  </si>
+  <si>
+    <t>Preferred source for FY2019 historical observations</t>
+  </si>
+  <si>
+    <t>SRC007</t>
+  </si>
+  <si>
+    <t>Zalando Annual Report 2019</t>
+  </si>
+  <si>
+    <t>zalando_annual_report_2019.pdf</t>
+  </si>
+  <si>
+    <t>FY2019 original reporting; historical definitions</t>
+  </si>
+  <si>
+    <t>Used for validation and definition-change research</t>
+  </si>
+  <si>
+    <t>comparison_period</t>
+  </si>
+  <si>
+    <t>Q1 2026</t>
+  </si>
+  <si>
+    <t>Q</t>
+  </si>
+  <si>
+    <t>Q1 2025</t>
+  </si>
+  <si>
+    <t>Zalando Quarterly Statement Q1 2026</t>
+  </si>
+  <si>
+    <t>Reported 2026 growth materially affected by ABOUT YOU consolidation; LTM customer KPIs include ABOUT YOU for full LTM</t>
+  </si>
+  <si>
+    <t>Q1 2024</t>
+  </si>
+  <si>
+    <t>Prior-year comparative as presented in Q1 2026 statement; ABOUT YOU not consolidated in Q1 2025</t>
+  </si>
+  <si>
+    <t>Q2 2026</t>
+  </si>
+  <si>
+    <t>Q2 2025</t>
+  </si>
+  <si>
+    <t>Zalando Half-Year Report 2026</t>
+  </si>
+  <si>
+    <t>Q2 figures not subject to review; LTM customer KPIs include ABOUT YOU for full LTM</t>
+  </si>
+  <si>
+    <t>Q2 2024</t>
+  </si>
+  <si>
+    <t>Prior-year comparative as presented in H1 2026 report; ABOUT YOU not consolidated in Q2 2025</t>
+  </si>
+  <si>
+    <t>H1 2026</t>
+  </si>
+  <si>
+    <t>H1</t>
+  </si>
+  <si>
+    <t>H1 2025</t>
+  </si>
+  <si>
+    <t>Reported H1 growth materially affected by ABOUT YOU consolidation; LTM customer KPIs include ABOUT YOU for full LTM</t>
+  </si>
+  <si>
+    <t>H1 2024</t>
+  </si>
+  <si>
+    <t>Prior-year comparative as presented in H1 2026 report; ABOUT YOU not consolidated in H1 2025</t>
   </si>
 </sst>
 </file>
@@ -587,7 +762,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>4</v>
@@ -602,16 +777,16 @@
         <v>6</v>
       </c>
       <c r="I1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J1" s="5" t="s">
         <v>26</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>27</v>
       </c>
       <c r="K1" s="5" t="s">
         <v>7</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M1" s="5" t="s">
         <v>8</v>
@@ -620,30 +795,30 @@
         <v>9</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="C2" s="5">
         <v>2025</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E2" s="5">
         <v>17560.2</v>
@@ -679,27 +854,27 @@
         <v>1877.4</v>
       </c>
       <c r="P2" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q2" s="5">
         <v>2</v>
       </c>
       <c r="R2" s="5" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="C3" s="5">
         <v>2025</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F3" s="5">
         <v>11278.7</v>
@@ -714,27 +889,27 @@
         <v>368.9</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q3" s="5">
         <v>83</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="C4" s="5">
         <v>2025</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F4" s="5">
         <v>1091.3</v>
@@ -749,27 +924,27 @@
         <v>17.7</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q4" s="5">
         <v>83</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C5" s="5">
         <v>2024</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E5" s="5">
         <v>15311.3</v>
@@ -805,27 +980,27 @@
         <v>2587.8000000000002</v>
       </c>
       <c r="P5" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q5" s="5">
         <v>2</v>
       </c>
       <c r="R5" s="5" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C6" s="5">
         <v>2024</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F6" s="5">
         <v>9657.7000000000007</v>
@@ -840,27 +1015,27 @@
         <v>394.2</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q6" s="5">
         <v>83</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C7" s="5">
         <v>2024</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F7" s="5">
         <v>952.6</v>
@@ -875,29 +1050,294 @@
         <v>-1.9</v>
       </c>
       <c r="P7" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Q7" s="5">
         <v>83</v>
       </c>
       <c r="R7" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A8" s="4"/>
+      <c r="A8" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="5">
+        <v>2023</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E8" s="5">
+        <v>14631</v>
+      </c>
+      <c r="F8" s="5">
+        <v>10143.1</v>
+      </c>
+      <c r="G8" s="5">
+        <v>349.9</v>
+      </c>
+      <c r="H8" s="5">
+        <v>3.5</v>
+      </c>
+      <c r="I8" s="5">
+        <v>190.9</v>
+      </c>
+      <c r="J8" s="5">
+        <v>1.9</v>
+      </c>
+      <c r="K8" s="5">
+        <v>-263.2</v>
+      </c>
+      <c r="L8" s="5">
+        <v>-441.8</v>
+      </c>
+      <c r="M8" s="5">
+        <v>949.5</v>
+      </c>
+      <c r="N8" s="5">
+        <v>683.8</v>
+      </c>
+      <c r="O8" s="5">
+        <v>2533.1999999999998</v>
+      </c>
+      <c r="P8" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q8" s="5">
+        <v>2</v>
+      </c>
+      <c r="R8" s="5" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A9" s="4"/>
+      <c r="A9" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="5">
+        <v>2022</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="5">
+        <v>14788.7</v>
+      </c>
+      <c r="F9" s="5">
+        <v>10344.799999999999</v>
+      </c>
+      <c r="G9" s="5">
+        <v>184.6</v>
+      </c>
+      <c r="H9" s="5">
+        <v>1.8</v>
+      </c>
+      <c r="I9" s="5">
+        <v>81</v>
+      </c>
+      <c r="J9" s="5">
+        <v>0.8</v>
+      </c>
+      <c r="K9" s="5">
+        <v>-351.7</v>
+      </c>
+      <c r="L9" s="5">
+        <v>-211.6</v>
+      </c>
+      <c r="M9" s="5">
+        <v>459.9</v>
+      </c>
+      <c r="N9" s="5">
+        <v>-18.8</v>
+      </c>
+      <c r="O9" s="5">
+        <v>2024.8</v>
+      </c>
+      <c r="P9" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q9" s="5">
+        <v>2</v>
+      </c>
+      <c r="R9" s="5" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A10" s="4"/>
+      <c r="A10" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="5">
+        <v>2021</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" s="5">
+        <v>14332.7</v>
+      </c>
+      <c r="F10" s="5">
+        <v>10354</v>
+      </c>
+      <c r="G10" s="5">
+        <v>468.4</v>
+      </c>
+      <c r="H10" s="5">
+        <v>4.5</v>
+      </c>
+      <c r="I10" s="5">
+        <v>424.7</v>
+      </c>
+      <c r="J10" s="5">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="K10" s="5">
+        <v>-332.9</v>
+      </c>
+      <c r="L10" s="5">
+        <v>-162.1</v>
+      </c>
+      <c r="M10" s="5">
+        <v>616.20000000000005</v>
+      </c>
+      <c r="N10" s="5">
+        <v>283.2</v>
+      </c>
+      <c r="O10" s="5">
+        <v>2287.9</v>
+      </c>
+      <c r="P10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q10" s="5">
+        <v>2</v>
+      </c>
+      <c r="R10" s="5" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A11" s="4"/>
+      <c r="A11" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" s="5">
+        <v>2020</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11" s="5">
+        <v>10696</v>
+      </c>
+      <c r="F11" s="5">
+        <v>7982</v>
+      </c>
+      <c r="G11" s="5">
+        <v>420.8</v>
+      </c>
+      <c r="H11" s="5">
+        <v>5.3</v>
+      </c>
+      <c r="I11" s="5">
+        <v>367</v>
+      </c>
+      <c r="J11" s="5">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="K11" s="5">
+        <v>-250</v>
+      </c>
+      <c r="L11" s="5">
+        <v>-87.4</v>
+      </c>
+      <c r="M11" s="5">
+        <v>527.4</v>
+      </c>
+      <c r="N11" s="5">
+        <v>284.5</v>
+      </c>
+      <c r="O11" s="5">
+        <v>2644</v>
+      </c>
+      <c r="P11" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q11" s="5">
+        <v>2</v>
+      </c>
+      <c r="R11" s="5" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A12" s="4"/>
+      <c r="A12" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="5">
+        <v>2019</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E12" s="5">
+        <v>8202.9</v>
+      </c>
+      <c r="F12" s="5">
+        <v>6482.5</v>
+      </c>
+      <c r="G12" s="5">
+        <v>224.9</v>
+      </c>
+      <c r="H12" s="5">
+        <v>3.5</v>
+      </c>
+      <c r="I12" s="5">
+        <v>165.8</v>
+      </c>
+      <c r="J12" s="5">
+        <v>2.6</v>
+      </c>
+      <c r="K12" s="5">
+        <v>-306.5</v>
+      </c>
+      <c r="L12" s="5">
+        <v>-147.69999999999999</v>
+      </c>
+      <c r="M12" s="5">
+        <v>327.2</v>
+      </c>
+      <c r="N12" s="5">
+        <v>41.6</v>
+      </c>
+      <c r="O12" s="5">
+        <v>976.5</v>
+      </c>
+      <c r="P12" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q12" s="5">
+        <v>2</v>
+      </c>
+      <c r="R12" s="5" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13" s="4"/>
@@ -957,39 +1397,39 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>13</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="C2" s="3">
         <v>2025</v>
@@ -1013,21 +1453,21 @@
         <v>16582</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K2" s="3">
         <v>2</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C3" s="3">
         <v>2024</v>
@@ -1051,29 +1491,201 @@
         <v>15309</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K3" s="3">
         <v>2</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A4" s="4"/>
+      <c r="A4" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="3">
+        <v>2023</v>
+      </c>
+      <c r="D4" s="3">
+        <v>49.6</v>
+      </c>
+      <c r="E4" s="3">
+        <v>244.8</v>
+      </c>
+      <c r="F4" s="3">
+        <v>295.2</v>
+      </c>
+      <c r="G4" s="3">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="H4" s="3">
+        <v>59.8</v>
+      </c>
+      <c r="I4" s="3">
+        <v>15793</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="K4" s="3">
+        <v>2</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5" s="4"/>
+      <c r="A5" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="3">
+        <v>2022</v>
+      </c>
+      <c r="D5" s="3">
+        <v>51.2</v>
+      </c>
+      <c r="E5" s="3">
+        <v>261.10000000000002</v>
+      </c>
+      <c r="F5" s="3">
+        <v>288.60000000000002</v>
+      </c>
+      <c r="G5" s="3">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="H5" s="3">
+        <v>56.6</v>
+      </c>
+      <c r="I5" s="3">
+        <v>16999</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K5" s="3">
+        <v>2</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" s="4"/>
+      <c r="A6" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="3">
+        <v>2021</v>
+      </c>
+      <c r="D6" s="3">
+        <v>48.5</v>
+      </c>
+      <c r="E6" s="3">
+        <v>252.2</v>
+      </c>
+      <c r="F6" s="3">
+        <v>295.60000000000002</v>
+      </c>
+      <c r="G6" s="3">
+        <v>5.2</v>
+      </c>
+      <c r="H6" s="3">
+        <v>56.8</v>
+      </c>
+      <c r="I6" s="3">
+        <v>16060</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="K6" s="3">
+        <v>2</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" s="4"/>
+      <c r="A7" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="3">
+        <v>2020</v>
+      </c>
+      <c r="D7" s="3">
+        <v>38.700000000000003</v>
+      </c>
+      <c r="E7" s="3">
+        <v>185.5</v>
+      </c>
+      <c r="F7" s="3">
+        <v>276.3</v>
+      </c>
+      <c r="G7" s="3">
+        <v>4.8</v>
+      </c>
+      <c r="H7" s="3">
+        <v>57.7</v>
+      </c>
+      <c r="I7" s="3">
+        <v>14194</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="K7" s="3">
+        <v>2</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="4"/>
+      <c r="A8" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="3">
+        <v>2019</v>
+      </c>
+      <c r="D8" s="3">
+        <v>31</v>
+      </c>
+      <c r="E8" s="3">
+        <v>144.9</v>
+      </c>
+      <c r="G8" s="3">
+        <v>4.7</v>
+      </c>
+      <c r="H8" s="3">
+        <v>56.6</v>
+      </c>
+      <c r="I8" s="3">
+        <v>13763</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="K8" s="3">
+        <v>2</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="4"/>
@@ -1096,87 +1708,660 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98BF5636-8179-9543-8900-484D288F4585}">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="9" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="17" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F1" t="s">
+        <v>40</v>
+      </c>
+      <c r="G1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="17" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F2" t="s">
+        <v>62</v>
+      </c>
+      <c r="G2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="17" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E3" t="s">
+        <v>65</v>
+      </c>
+      <c r="F3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="17" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4" t="s">
+        <v>69</v>
+      </c>
+      <c r="F4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="17" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" t="s">
+        <v>73</v>
+      </c>
+      <c r="F5" t="s">
+        <v>74</v>
+      </c>
+      <c r="G5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="17" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F6" t="s">
+        <v>78</v>
+      </c>
+      <c r="G6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="17" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" t="s">
+        <v>81</v>
+      </c>
+      <c r="F7" t="s">
+        <v>82</v>
+      </c>
+      <c r="G7" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="17" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B8" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" t="s">
+        <v>85</v>
+      </c>
+      <c r="D8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" t="s">
+        <v>86</v>
+      </c>
+      <c r="F8" t="s">
+        <v>87</v>
+      </c>
+      <c r="G8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3EA10AC5-5D6D-A948-92DF-1B9FC6B2EF51}">
+  <dimension ref="A1:U7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J1" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1" t="s">
+        <v>7</v>
+      </c>
+      <c r="L1" t="s">
+        <v>14</v>
+      </c>
+      <c r="M1" t="s">
+        <v>15</v>
+      </c>
+      <c r="N1" t="s">
+        <v>30</v>
+      </c>
+      <c r="O1" t="s">
+        <v>31</v>
+      </c>
+      <c r="P1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E1" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H1" t="s">
-        <v>44</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="Q1" t="s">
+        <v>8</v>
+      </c>
+      <c r="R1" t="s">
+        <v>9</v>
+      </c>
+      <c r="S1" t="s">
+        <v>11</v>
+      </c>
+      <c r="T1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" ht="17" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>45</v>
+      <c r="U1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>90</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" t="s">
-        <v>30</v>
+        <v>91</v>
+      </c>
+      <c r="C2">
+        <v>2026</v>
       </c>
       <c r="D2" t="s">
-        <v>46</v>
-      </c>
-      <c r="E2" s="6">
-        <v>46093</v>
-      </c>
-      <c r="F2" t="s">
-        <v>47</v>
-      </c>
-      <c r="G2" t="s">
-        <v>48</v>
-      </c>
-      <c r="H2" t="s">
-        <v>49</v>
-      </c>
-      <c r="I2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="17" x14ac:dyDescent="0.25">
-      <c r="A3" s="1"/>
-    </row>
-    <row r="4" spans="1:9" ht="17" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" ht="17" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-    </row>
-    <row r="6" spans="1:9" ht="17" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-    </row>
-    <row r="7" spans="1:9" ht="17" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-    </row>
-    <row r="8" spans="1:9" ht="17" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
+        <v>92</v>
+      </c>
+      <c r="E2">
+        <v>4294.3</v>
+      </c>
+      <c r="F2">
+        <v>2996.1</v>
+      </c>
+      <c r="G2">
+        <v>64.8</v>
+      </c>
+      <c r="H2">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="I2">
+        <v>-79.7</v>
+      </c>
+      <c r="J2">
+        <v>-2.7</v>
+      </c>
+      <c r="K2">
+        <v>-69.7</v>
+      </c>
+      <c r="L2">
+        <v>62.3</v>
+      </c>
+      <c r="M2">
+        <v>69.5</v>
+      </c>
+      <c r="N2">
+        <v>305.2</v>
+      </c>
+      <c r="O2">
+        <v>4.8</v>
+      </c>
+      <c r="P2">
+        <v>63.1</v>
+      </c>
+      <c r="Q2">
+        <v>-438.2</v>
+      </c>
+      <c r="R2">
+        <v>-512.9</v>
+      </c>
+      <c r="S2" t="s">
+        <v>93</v>
+      </c>
+      <c r="T2">
+        <v>2</v>
+      </c>
+      <c r="U2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3">
+        <v>2025</v>
+      </c>
+      <c r="D3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E3">
+        <v>3528.4</v>
+      </c>
+      <c r="F3">
+        <v>2419.5</v>
+      </c>
+      <c r="G3">
+        <v>46.7</v>
+      </c>
+      <c r="H3">
+        <v>1.9</v>
+      </c>
+      <c r="I3">
+        <v>21.4</v>
+      </c>
+      <c r="J3">
+        <v>0.9</v>
+      </c>
+      <c r="K3">
+        <v>-33.6</v>
+      </c>
+      <c r="L3">
+        <v>52.4</v>
+      </c>
+      <c r="M3">
+        <v>58.5</v>
+      </c>
+      <c r="N3">
+        <v>296.7</v>
+      </c>
+      <c r="O3">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="P3">
+        <v>61.2</v>
+      </c>
+      <c r="Q3">
+        <v>-143</v>
+      </c>
+      <c r="R3">
+        <v>-192.1</v>
+      </c>
+      <c r="S3" t="s">
+        <v>93</v>
+      </c>
+      <c r="T3">
+        <v>2</v>
+      </c>
+      <c r="U3" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C4">
+        <v>2026</v>
+      </c>
+      <c r="D4" t="s">
+        <v>98</v>
+      </c>
+      <c r="E4">
+        <v>4915</v>
+      </c>
+      <c r="F4">
+        <v>3424.4</v>
+      </c>
+      <c r="G4">
+        <v>204.8</v>
+      </c>
+      <c r="H4">
+        <v>6</v>
+      </c>
+      <c r="I4">
+        <v>111.1</v>
+      </c>
+      <c r="J4">
+        <v>3.2</v>
+      </c>
+      <c r="K4">
+        <v>-54.7</v>
+      </c>
+      <c r="L4">
+        <v>62.5</v>
+      </c>
+      <c r="M4">
+        <v>77.5</v>
+      </c>
+      <c r="N4">
+        <v>307</v>
+      </c>
+      <c r="O4">
+        <v>4.8</v>
+      </c>
+      <c r="P4">
+        <v>63.4</v>
+      </c>
+      <c r="Q4">
+        <v>473.3</v>
+      </c>
+      <c r="R4">
+        <v>417.9</v>
+      </c>
+      <c r="S4" t="s">
+        <v>99</v>
+      </c>
+      <c r="T4">
+        <v>2</v>
+      </c>
+      <c r="U4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5">
+        <v>2025</v>
+      </c>
+      <c r="D5" t="s">
+        <v>101</v>
+      </c>
+      <c r="E5">
+        <v>4073.4</v>
+      </c>
+      <c r="F5">
+        <v>2835.1</v>
+      </c>
+      <c r="G5">
+        <v>185.5</v>
+      </c>
+      <c r="H5">
+        <v>6.5</v>
+      </c>
+      <c r="I5">
+        <v>145.19999999999999</v>
+      </c>
+      <c r="J5">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="K5">
+        <v>-59.8</v>
+      </c>
+      <c r="L5">
+        <v>52.9</v>
+      </c>
+      <c r="M5">
+        <v>65</v>
+      </c>
+      <c r="N5">
+        <v>298.3</v>
+      </c>
+      <c r="O5">
+        <v>4.8</v>
+      </c>
+      <c r="P5">
+        <v>61.6</v>
+      </c>
+      <c r="Q5">
+        <v>283.8</v>
+      </c>
+      <c r="R5">
+        <v>209.3</v>
+      </c>
+      <c r="S5" t="s">
+        <v>99</v>
+      </c>
+      <c r="T5">
+        <v>2</v>
+      </c>
+      <c r="U5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C6">
+        <v>2026</v>
+      </c>
+      <c r="D6" t="s">
+        <v>105</v>
+      </c>
+      <c r="E6">
+        <v>9199.7000000000007</v>
+      </c>
+      <c r="F6">
+        <v>6420.6</v>
+      </c>
+      <c r="G6">
+        <v>269.60000000000002</v>
+      </c>
+      <c r="H6">
+        <v>4.2</v>
+      </c>
+      <c r="I6">
+        <v>31.4</v>
+      </c>
+      <c r="J6">
+        <v>0.5</v>
+      </c>
+      <c r="K6">
+        <v>-124.4</v>
+      </c>
+      <c r="L6">
+        <v>62.5</v>
+      </c>
+      <c r="M6">
+        <v>146.9</v>
+      </c>
+      <c r="N6">
+        <v>307</v>
+      </c>
+      <c r="O6">
+        <v>4.8</v>
+      </c>
+      <c r="P6">
+        <v>63.4</v>
+      </c>
+      <c r="Q6">
+        <v>35.1</v>
+      </c>
+      <c r="R6">
+        <v>-95</v>
+      </c>
+      <c r="S6" t="s">
+        <v>99</v>
+      </c>
+      <c r="T6">
+        <v>2</v>
+      </c>
+      <c r="U6" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" t="s">
+        <v>104</v>
+      </c>
+      <c r="C7">
+        <v>2025</v>
+      </c>
+      <c r="D7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E7">
+        <v>7601.8</v>
+      </c>
+      <c r="F7">
+        <v>5254.6</v>
+      </c>
+      <c r="G7">
+        <v>232.3</v>
+      </c>
+      <c r="H7">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="I7">
+        <v>166.6</v>
+      </c>
+      <c r="J7">
+        <v>3.2</v>
+      </c>
+      <c r="K7">
+        <v>-93.4</v>
+      </c>
+      <c r="L7">
+        <v>52.9</v>
+      </c>
+      <c r="M7">
+        <v>123.5</v>
+      </c>
+      <c r="N7">
+        <v>298.3</v>
+      </c>
+      <c r="O7">
+        <v>4.8</v>
+      </c>
+      <c r="P7">
+        <v>61.6</v>
+      </c>
+      <c r="Q7">
+        <v>140.80000000000001</v>
+      </c>
+      <c r="R7">
+        <v>17.2</v>
+      </c>
+      <c r="S7" t="s">
+        <v>99</v>
+      </c>
+      <c r="T7">
+        <v>2</v>
+      </c>
+      <c r="U7" t="s">
+        <v>108</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>